<commit_message>
feat(r6): add ticker→name company_dim seed/table + fix 2412 canonical name
Names live only in the R6 ontology (fact tables store ticker only). This
lands a canonical ticker→company dimension so RAG metadata/reports can JOIN
instead of hardcoding name mappings.

- docs/r6/ontology/seeds/company_dim.csv: 20-company seed (SSOT, generated
  from Ontology_V1 02_company公司; join key = ticker per V1_1_JOIN_KEY_TICKER)
- migrations/2026-06-17_create_company_dim.sql: CREATE OR REPLACE TABLE
  polaris_core.company_dim + inline INSERT (20 rows) + post-apply checks.
  NOT executed — applied by R1/R4 via SOP §7 (BQ_ALLOW_CORE_WRITE=1).
- Ontology_V1.xlsx: reverse ticker=2412 canonical name 中華電信→中華電
  (中華電信 kept as alias); updated 02/08/09/00_readme/12_governance and
  appended a 99_change_log reversal row. History rows + external Question
  Bank references left untouched.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/r6/ontology/Ontology_V1.xlsx
+++ b/docs/r6/ontology/Ontology_V1.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="25600" windowHeight="14140" tabRatio="600" firstSheet="2" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_readme" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_industry產業" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_company公司" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_financial_metric財務指標" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_compliance_terms法遵名詞" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_disclosure_events事件" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_theme" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_risk_signal" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_company_theme_mapping" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_company_industry_mapping" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_news_source_whitelist" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_quality_checks" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_source_taxonomy_mapping" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_governance_decisions" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_traceability_matrix" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_revenue_metrics_extension" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_revenue_field_matrix" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="99_change_log" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="00_readme" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="01_industry產業" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="02_company公司" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="03_financial_metric財務指標" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="05_compliance_terms法遵名詞" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="04_disclosure_events事件" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="06_theme" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="07_risk_signal" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="08_company_theme_mapping" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="09_company_industry_mapping" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="10_news_source_whitelist" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="11_quality_checks" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="12_source_taxonomy_mapping" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="12_governance_decisions" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="13_traceability_matrix" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="14_revenue_metrics_extension" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="15_revenue_field_matrix" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="99_change_log" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00_readme'!$A$1:$B$34</definedName>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>company_name is the canonical display name. For ticker=2412, company_name=中華電信 and aliases include 中華電, Chunghwa Telecom, 2412.</t>
+          <t>company_name is the canonical display name. For ticker=2412, company_name=中華電 and aliases include 中華電信, Chunghwa Telecom, 2412.</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>中華電信</t>
+          <t>中華電</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2447,7 +2447,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>中華電信</t>
+          <t>中華電</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>ticker=2412 canonical company_name is 中華電信; 中華電 is retained as alias.</t>
+          <t>ticker=2412 canonical company_name is 中華電; 中華電信 is retained as alias. (Reversed 2026-06-17 from prior 中華電信 canonical — see 99_change_log.)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -5704,7 +5704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6066,6 +6066,23 @@
       <c r="C21" t="inlineStr">
         <is>
           <t>Added revenue cumulative metrics and revenue delta metrics. Standardized revenue storage unit: currency=TWD; unit=TWD_thousand. Supports Monthly Revenue Analysis, Financial QA, RAG Retrieval, and Revenue Trend Evaluation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TICKER_2412_CANONICAL_REVERSAL</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Reversed ticker=2412 canonical company_name 中華電信 -&gt; 中華電; 中華電信 retained as alias. Updated 02_company, 08/09 mappings, 00_readme, 12_governance_decisions. External Question Bank references (12/13) still use 中華電信 and were left unchanged.</t>
         </is>
       </c>
     </row>
@@ -7868,7 +7885,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>中華電信</t>
+          <t>中華電</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -7914,7 +7931,7 @@
       <c r="L12" s="8" t="n"/>
       <c r="M12" s="8" t="inlineStr">
         <is>
-          <t>中華電信,中華電,Chunghwa Telecom,2412</t>
+          <t>中華電信,Chunghwa Telecom,2412</t>
         </is>
       </c>
       <c r="N12" s="8" t="inlineStr">
@@ -14835,7 +14852,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>中華電信</t>
+          <t>中華電</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -14875,7 +14892,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>中華電信</t>
+          <t>中華電</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -14915,7 +14932,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>中華電信</t>
+          <t>中華電</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(r6): add ticker→name company_dim seed/table + fix 2412 canonical name (#84)
Names live only in the R6 ontology (fact tables store ticker only). This
lands a canonical ticker→company dimension so RAG metadata/reports can JOIN
instead of hardcoding name mappings.

- docs/r6/ontology/seeds/company_dim.csv: 20-company seed (SSOT, generated
  from Ontology_V1 02_company公司; join key = ticker per V1_1_JOIN_KEY_TICKER)
- migrations/2026-06-17_create_company_dim.sql: CREATE OR REPLACE TABLE
  polaris_core.company_dim + inline INSERT (20 rows) + post-apply checks.
  NOT executed — applied by R1/R4 via SOP §7 (BQ_ALLOW_CORE_WRITE=1).
- Ontology_V1.xlsx: reverse ticker=2412 canonical name 中華電信→中華電
  (中華電信 kept as alias); updated 02/08/09/00_readme/12_governance and
  appended a 99_change_log reversal row. History rows + external Question
  Bank references left untouched.

Co-authored-by: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/r6/ontology/Ontology_V1.xlsx
+++ b/docs/r6/ontology/Ontology_V1.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="25600" windowHeight="14140" tabRatio="600" firstSheet="2" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_readme" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_industry產業" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_company公司" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_financial_metric財務指標" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_compliance_terms法遵名詞" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_disclosure_events事件" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_theme" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_risk_signal" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_company_theme_mapping" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_company_industry_mapping" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_news_source_whitelist" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_quality_checks" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_source_taxonomy_mapping" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_governance_decisions" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_traceability_matrix" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_revenue_metrics_extension" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_revenue_field_matrix" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="99_change_log" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="00_readme" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="01_industry產業" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="02_company公司" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="03_financial_metric財務指標" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="05_compliance_terms法遵名詞" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="04_disclosure_events事件" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="06_theme" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="07_risk_signal" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="08_company_theme_mapping" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="09_company_industry_mapping" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="10_news_source_whitelist" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="11_quality_checks" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="12_source_taxonomy_mapping" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="12_governance_decisions" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="13_traceability_matrix" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="14_revenue_metrics_extension" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="15_revenue_field_matrix" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="99_change_log" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00_readme'!$A$1:$B$34</definedName>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>company_name is the canonical display name. For ticker=2412, company_name=中華電信 and aliases include 中華電, Chunghwa Telecom, 2412.</t>
+          <t>company_name is the canonical display name. For ticker=2412, company_name=中華電 and aliases include 中華電信, Chunghwa Telecom, 2412.</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>中華電信</t>
+          <t>中華電</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2447,7 +2447,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>中華電信</t>
+          <t>中華電</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>ticker=2412 canonical company_name is 中華電信; 中華電 is retained as alias.</t>
+          <t>ticker=2412 canonical company_name is 中華電; 中華電信 is retained as alias. (Reversed 2026-06-17 from prior 中華電信 canonical — see 99_change_log.)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -5704,7 +5704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6066,6 +6066,23 @@
       <c r="C21" t="inlineStr">
         <is>
           <t>Added revenue cumulative metrics and revenue delta metrics. Standardized revenue storage unit: currency=TWD; unit=TWD_thousand. Supports Monthly Revenue Analysis, Financial QA, RAG Retrieval, and Revenue Trend Evaluation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TICKER_2412_CANONICAL_REVERSAL</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Reversed ticker=2412 canonical company_name 中華電信 -&gt; 中華電; 中華電信 retained as alias. Updated 02_company, 08/09 mappings, 00_readme, 12_governance_decisions. External Question Bank references (12/13) still use 中華電信 and were left unchanged.</t>
         </is>
       </c>
     </row>
@@ -7868,7 +7885,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>中華電信</t>
+          <t>中華電</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -7914,7 +7931,7 @@
       <c r="L12" s="8" t="n"/>
       <c r="M12" s="8" t="inlineStr">
         <is>
-          <t>中華電信,中華電,Chunghwa Telecom,2412</t>
+          <t>中華電信,Chunghwa Telecom,2412</t>
         </is>
       </c>
       <c r="N12" s="8" t="inlineStr">
@@ -14835,7 +14852,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>中華電信</t>
+          <t>中華電</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -14875,7 +14892,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>中華電信</t>
+          <t>中華電</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -14915,7 +14932,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>中華電信</t>
+          <t>中華電</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs(r6): update source key and quarter table
</commit_message>
<xml_diff>
--- a/docs/r6/ontology/Ontology_V1.xlsx
+++ b/docs/r6/ontology/Ontology_V1.xlsx
@@ -1,29 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="25600" windowHeight="14140" tabRatio="600" firstSheet="2" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="00_readme" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="01_industry產業" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="02_company公司" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="03_financial_metric財務指標" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="05_compliance_terms法遵名詞" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="04_disclosure_events事件" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="06_theme" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="07_risk_signal" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="08_company_theme_mapping" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="09_company_industry_mapping" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="10_news_source_whitelist" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="11_quality_checks" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="12_source_taxonomy_mapping" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="12_governance_decisions" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="13_traceability_matrix" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="14_revenue_metrics_extension" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="15_revenue_field_matrix" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="99_change_log" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_readme" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_industry產業" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_company公司" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_financial_metric財務指標" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_compliance_terms法遵名詞" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_disclosure_events事件" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_theme" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_risk_signal" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_company_theme_mapping" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_company_industry_mapping" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_news_source_whitelist" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_quality_checks" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_source_taxonomy_mapping" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_governance_decisions" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_traceability_matrix" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_revenue_metrics_extension" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_revenue_field_matrix" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_quarter_table" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="99_change_log" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00_readme'!$A$1:$B$34</definedName>
@@ -35,7 +36,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'13_traceability_matrix'!$A$1:$H$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'14_revenue_metrics_extension'!$A$1:$M$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'15_revenue_field_matrix'!$A$1:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'99_change_log'!$A$1:$C$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'99_change_log'!$A$1:$C$21</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -69,7 +70,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -116,8 +117,13 @@
         <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005B3F8C"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="16">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -306,12 +312,26 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -447,6 +467,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2614,7 +2640,7 @@
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>source_id</t>
+          <t>source_key</t>
         </is>
       </c>
       <c r="B1" s="30" t="inlineStr">
@@ -5704,7 +5730,613 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:J13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="56" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="47" t="inlineStr">
+        <is>
+          <t>fiscal_period</t>
+        </is>
+      </c>
+      <c r="B1" s="47" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="C1" s="47" t="inlineStr">
+        <is>
+          <t>quarter</t>
+        </is>
+      </c>
+      <c r="D1" s="47" t="inlineStr">
+        <is>
+          <t>yyyyqq</t>
+        </is>
+      </c>
+      <c r="E1" s="47" t="inlineStr">
+        <is>
+          <t>quarter_start_month</t>
+        </is>
+      </c>
+      <c r="F1" s="47" t="inlineStr">
+        <is>
+          <t>quarter_end_month</t>
+        </is>
+      </c>
+      <c r="G1" s="47" t="inlineStr">
+        <is>
+          <t>start_date</t>
+        </is>
+      </c>
+      <c r="H1" s="47" t="inlineStr">
+        <is>
+          <t>end_date</t>
+        </is>
+      </c>
+      <c r="I1" s="47" t="inlineStr">
+        <is>
+          <t>month_keys</t>
+        </is>
+      </c>
+      <c r="J1" s="47" t="inlineStr">
+        <is>
+          <t>r6_notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="48" t="inlineStr">
+        <is>
+          <t>2024Q1</t>
+        </is>
+      </c>
+      <c r="B2" s="48" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C2" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="48" t="inlineStr">
+        <is>
+          <t>202401</t>
+        </is>
+      </c>
+      <c r="E2" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="G2" s="48" t="inlineStr">
+        <is>
+          <t>2024-01-01</t>
+        </is>
+      </c>
+      <c r="H2" s="48" t="inlineStr">
+        <is>
+          <t>2024-03-31</t>
+        </is>
+      </c>
+      <c r="I2" s="48" t="inlineStr">
+        <is>
+          <t>202401,202402,202403</t>
+        </is>
+      </c>
+      <c r="J2" s="48" t="inlineStr">
+        <is>
+          <t>Q1 對應 1–3 月，用於法說會、月營收與財務資料期間對齊。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="48" t="inlineStr">
+        <is>
+          <t>2024Q2</t>
+        </is>
+      </c>
+      <c r="B3" s="48" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C3" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="48" t="inlineStr">
+        <is>
+          <t>202402</t>
+        </is>
+      </c>
+      <c r="E3" s="48" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" s="48" t="n">
+        <v>6</v>
+      </c>
+      <c r="G3" s="48" t="inlineStr">
+        <is>
+          <t>2024-04-01</t>
+        </is>
+      </c>
+      <c r="H3" s="48" t="inlineStr">
+        <is>
+          <t>2024-06-30</t>
+        </is>
+      </c>
+      <c r="I3" s="48" t="inlineStr">
+        <is>
+          <t>202404,202405,202406</t>
+        </is>
+      </c>
+      <c r="J3" s="48" t="inlineStr">
+        <is>
+          <t>Q2 對應 4–6 月，用於法說會、月營收與財務資料期間對齊。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="48" t="inlineStr">
+        <is>
+          <t>2024Q3</t>
+        </is>
+      </c>
+      <c r="B4" s="48" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C4" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="48" t="inlineStr">
+        <is>
+          <t>202403</t>
+        </is>
+      </c>
+      <c r="E4" s="48" t="n">
+        <v>7</v>
+      </c>
+      <c r="F4" s="48" t="n">
+        <v>9</v>
+      </c>
+      <c r="G4" s="48" t="inlineStr">
+        <is>
+          <t>2024-07-01</t>
+        </is>
+      </c>
+      <c r="H4" s="48" t="inlineStr">
+        <is>
+          <t>2024-09-30</t>
+        </is>
+      </c>
+      <c r="I4" s="48" t="inlineStr">
+        <is>
+          <t>202407,202408,202409</t>
+        </is>
+      </c>
+      <c r="J4" s="48" t="inlineStr">
+        <is>
+          <t>Q3 對應 7–9 月，用於法說會、月營收與財務資料期間對齊。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="48" t="inlineStr">
+        <is>
+          <t>2024Q4</t>
+        </is>
+      </c>
+      <c r="B5" s="48" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C5" s="48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="48" t="inlineStr">
+        <is>
+          <t>202404</t>
+        </is>
+      </c>
+      <c r="E5" s="48" t="n">
+        <v>10</v>
+      </c>
+      <c r="F5" s="48" t="n">
+        <v>12</v>
+      </c>
+      <c r="G5" s="48" t="inlineStr">
+        <is>
+          <t>2024-10-01</t>
+        </is>
+      </c>
+      <c r="H5" s="48" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="I5" s="48" t="inlineStr">
+        <is>
+          <t>202410,202411,202412</t>
+        </is>
+      </c>
+      <c r="J5" s="48" t="inlineStr">
+        <is>
+          <t>Q4 對應 10–12 月，用於法說會、月營收與財務資料期間對齊。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="48" t="inlineStr">
+        <is>
+          <t>2025Q1</t>
+        </is>
+      </c>
+      <c r="B6" s="48" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C6" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="48" t="inlineStr">
+        <is>
+          <t>202501</t>
+        </is>
+      </c>
+      <c r="E6" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" s="48" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H6" s="48" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="I6" s="48" t="inlineStr">
+        <is>
+          <t>202501,202502,202503</t>
+        </is>
+      </c>
+      <c r="J6" s="48" t="inlineStr">
+        <is>
+          <t>Q1 對應 1–3 月，用於法說會、月營收與財務資料期間對齊。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="48" t="inlineStr">
+        <is>
+          <t>2025Q2</t>
+        </is>
+      </c>
+      <c r="B7" s="48" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C7" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="48" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="E7" s="48" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" s="48" t="n">
+        <v>6</v>
+      </c>
+      <c r="G7" s="48" t="inlineStr">
+        <is>
+          <t>2025-04-01</t>
+        </is>
+      </c>
+      <c r="H7" s="48" t="inlineStr">
+        <is>
+          <t>2025-06-30</t>
+        </is>
+      </c>
+      <c r="I7" s="48" t="inlineStr">
+        <is>
+          <t>202504,202505,202506</t>
+        </is>
+      </c>
+      <c r="J7" s="48" t="inlineStr">
+        <is>
+          <t>Q2 對應 4–6 月，用於法說會、月營收與財務資料期間對齊。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="48" t="inlineStr">
+        <is>
+          <t>2025Q3</t>
+        </is>
+      </c>
+      <c r="B8" s="48" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C8" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" s="48" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="E8" s="48" t="n">
+        <v>7</v>
+      </c>
+      <c r="F8" s="48" t="n">
+        <v>9</v>
+      </c>
+      <c r="G8" s="48" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="H8" s="48" t="inlineStr">
+        <is>
+          <t>2025-09-30</t>
+        </is>
+      </c>
+      <c r="I8" s="48" t="inlineStr">
+        <is>
+          <t>202507,202508,202509</t>
+        </is>
+      </c>
+      <c r="J8" s="48" t="inlineStr">
+        <is>
+          <t>Q3 對應 7–9 月，用於法說會、月營收與財務資料期間對齊。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="48" t="inlineStr">
+        <is>
+          <t>2025Q4</t>
+        </is>
+      </c>
+      <c r="B9" s="48" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C9" s="48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="48" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="E9" s="48" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" s="48" t="n">
+        <v>12</v>
+      </c>
+      <c r="G9" s="48" t="inlineStr">
+        <is>
+          <t>2025-10-01</t>
+        </is>
+      </c>
+      <c r="H9" s="48" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="I9" s="48" t="inlineStr">
+        <is>
+          <t>202510,202511,202512</t>
+        </is>
+      </c>
+      <c r="J9" s="48" t="inlineStr">
+        <is>
+          <t>Q4 對應 10–12 月，用於法說會、月營收與財務資料期間對齊。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="48" t="inlineStr">
+        <is>
+          <t>2026Q1</t>
+        </is>
+      </c>
+      <c r="B10" s="48" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C10" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="48" t="inlineStr">
+        <is>
+          <t>202601</t>
+        </is>
+      </c>
+      <c r="E10" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" s="48" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H10" s="48" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="I10" s="48" t="inlineStr">
+        <is>
+          <t>202601,202602,202603</t>
+        </is>
+      </c>
+      <c r="J10" s="48" t="inlineStr">
+        <is>
+          <t>Q1 對應 1–3 月，用於法說會、月營收與財務資料期間對齊。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="48" t="inlineStr">
+        <is>
+          <t>2026Q2</t>
+        </is>
+      </c>
+      <c r="B11" s="48" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C11" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="48" t="inlineStr">
+        <is>
+          <t>202602</t>
+        </is>
+      </c>
+      <c r="E11" s="48" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" s="48" t="n">
+        <v>6</v>
+      </c>
+      <c r="G11" s="48" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="H11" s="48" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="I11" s="48" t="inlineStr">
+        <is>
+          <t>202604,202605,202606</t>
+        </is>
+      </c>
+      <c r="J11" s="48" t="inlineStr">
+        <is>
+          <t>Q2 對應 4–6 月，用於法說會、月營收與財務資料期間對齊。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="48" t="inlineStr">
+        <is>
+          <t>2026Q3</t>
+        </is>
+      </c>
+      <c r="B12" s="48" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C12" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" s="48" t="inlineStr">
+        <is>
+          <t>202603</t>
+        </is>
+      </c>
+      <c r="E12" s="48" t="n">
+        <v>7</v>
+      </c>
+      <c r="F12" s="48" t="n">
+        <v>9</v>
+      </c>
+      <c r="G12" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="H12" s="48" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I12" s="48" t="inlineStr">
+        <is>
+          <t>202607,202608,202609</t>
+        </is>
+      </c>
+      <c r="J12" s="48" t="inlineStr">
+        <is>
+          <t>Q3 對應 7–9 月，用於法說會、月營收與財務資料期間對齊。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="48" t="inlineStr">
+        <is>
+          <t>2026Q4</t>
+        </is>
+      </c>
+      <c r="B13" s="48" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C13" s="48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" s="48" t="inlineStr">
+        <is>
+          <t>202604</t>
+        </is>
+      </c>
+      <c r="E13" s="48" t="n">
+        <v>10</v>
+      </c>
+      <c r="F13" s="48" t="n">
+        <v>12</v>
+      </c>
+      <c r="G13" s="48" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="H13" s="48" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="I13" s="48" t="inlineStr">
+        <is>
+          <t>202610,202611,202612</t>
+        </is>
+      </c>
+      <c r="J13" s="48" t="inlineStr">
+        <is>
+          <t>Q4 對應 10–12 月，用於法說會、月營收與財務資料期間對齊。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6083,6 +6715,23 @@
       <c r="C22" t="inlineStr">
         <is>
           <t>Reversed ticker=2412 canonical company_name 中華電信 -&gt; 中華電; 中華電信 retained as alias. Updated 02_company, 08/09 mappings, 00_readme, 12_governance_decisions. External Question Bank references (12/13) still use 中華電信 and were left unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SOURCE_KEY_AND_QUARTER_TABLE</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Renamed 10_news_source_whitelist.source_id to source_key for R4 source mapping alignment; added 16_quarter_table covering 2024Q1 through 2026Q4 with fiscal_period/year/quarter/yyyyqq/start_date/end_date/month_keys mapping.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(r6): update disclosure events and news sources
</commit_message>
<xml_diff>
--- a/docs/r6/ontology/Ontology_V1.xlsx
+++ b/docs/r6/ontology/Ontology_V1.xlsx
@@ -29,8 +29,10 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00_readme'!$A$1:$B$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_financial_metric財務指標'!$A$1:$K$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'04_disclosure_events事件'!$A$1:$K$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'08_company_theme_mapping'!$A$1:$H$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'09_company_industry_mapping'!$A$1:$L$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'10_news_source_whitelist'!$A$1:$H$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'12_source_taxonomy_mapping'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'12_governance_decisions'!$A$1:$I$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'13_traceability_matrix'!$A$1:$H$5</definedName>
@@ -70,7 +72,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -120,6 +122,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="005B3F8C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005B3F91"/>
       </patternFill>
     </fill>
   </fills>
@@ -331,7 +338,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -473,6 +480,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2622,610 +2638,695 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col width="27" customWidth="1" style="1" min="1" max="1"/>
-    <col width="26" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
-    <col width="12" bestFit="1" customWidth="1" style="1" min="3" max="3"/>
-    <col width="13" bestFit="1" customWidth="1" style="1" min="4" max="4"/>
-    <col width="16" customWidth="1" style="1" min="5" max="5"/>
+    <col width="26" customWidth="1" style="1" min="1" max="1"/>
+    <col width="24" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
+    <col width="16" bestFit="1" customWidth="1" style="1" min="3" max="3"/>
+    <col width="18" bestFit="1" customWidth="1" style="1" min="4" max="4"/>
+    <col width="28" customWidth="1" style="1" min="5" max="5"/>
     <col width="18" bestFit="1" customWidth="1" style="1" min="6" max="6"/>
-    <col width="27" customWidth="1" style="1" min="7" max="7"/>
-    <col width="19" customWidth="1" style="1" min="8" max="8"/>
+    <col width="42" customWidth="1" style="1" min="7" max="7"/>
+    <col width="18" customWidth="1" style="1" min="8" max="8"/>
     <col width="8.83203125" customWidth="1" style="1" min="9" max="13"/>
     <col width="8.83203125" customWidth="1" style="1" min="14" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="30" t="inlineStr">
+      <c r="A1" s="50" t="inlineStr">
         <is>
           <t>source_key</t>
         </is>
       </c>
-      <c r="B1" s="30" t="inlineStr">
+      <c r="B1" s="50" t="inlineStr">
         <is>
           <t>source_name</t>
         </is>
       </c>
-      <c r="C1" s="30" t="inlineStr">
+      <c r="C1" s="50" t="inlineStr">
         <is>
           <t>trust_tier</t>
         </is>
       </c>
-      <c r="D1" s="30" t="inlineStr">
+      <c r="D1" s="50" t="inlineStr">
         <is>
           <t>source_type</t>
         </is>
       </c>
-      <c r="E1" s="30" t="inlineStr">
+      <c r="E1" s="50" t="inlineStr">
         <is>
           <t>use_case</t>
         </is>
       </c>
-      <c r="F1" s="30" t="inlineStr">
+      <c r="F1" s="50" t="inlineStr">
         <is>
           <t>allowed_for_fact</t>
         </is>
       </c>
-      <c r="G1" s="30" t="inlineStr">
+      <c r="G1" s="50" t="inlineStr">
         <is>
           <t>r6_note</t>
         </is>
       </c>
-      <c r="H1" s="31" t="inlineStr">
+      <c r="H1" s="49" t="inlineStr">
         <is>
           <t>citation_required</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="51" t="inlineStr">
         <is>
           <t>PRIMARY_MOPS</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="51" t="inlineStr">
         <is>
           <t>公開資訊觀測站</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
+      <c r="C2" s="51" t="inlineStr">
         <is>
           <t>Primary</t>
         </is>
       </c>
-      <c r="D2" s="11" t="inlineStr">
+      <c r="D2" s="51" t="inlineStr">
         <is>
           <t>MOPS</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
+      <c r="E2" s="51" t="inlineStr">
         <is>
           <t>公告/重大訊息/財報</t>
         </is>
       </c>
-      <c r="F2" s="11" t="inlineStr">
+      <c r="F2" s="51" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G2" s="11" t="inlineStr">
+      <c r="G2" s="51" t="inlineStr">
         <is>
           <t>官方一手來源，最高優先</t>
         </is>
       </c>
-      <c r="H2" s="12" t="inlineStr">
+      <c r="H2" s="48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="51" t="inlineStr">
         <is>
           <t>PRIMARY_TWSE</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="51" t="inlineStr">
         <is>
           <t>臺灣證券交易所</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="51" t="inlineStr">
         <is>
           <t>Primary</t>
         </is>
       </c>
-      <c r="D3" s="11" t="inlineStr">
+      <c r="D3" s="51" t="inlineStr">
         <is>
           <t>TWSE</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
+      <c r="E3" s="51" t="inlineStr">
         <is>
           <t>上市公司資訊/指數/交易制度</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr">
+      <c r="F3" s="51" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G3" s="11" t="inlineStr">
+      <c r="G3" s="51" t="inlineStr">
         <is>
           <t>官方一手來源</t>
         </is>
       </c>
-      <c r="H3" s="12" t="inlineStr">
+      <c r="H3" s="48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="51" t="inlineStr">
         <is>
           <t>PRIMARY_TPEX</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="51" t="inlineStr">
         <is>
           <t>櫃買中心</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="51" t="inlineStr">
         <is>
           <t>Primary</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="51" t="inlineStr">
         <is>
           <t>TPEx</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="51" t="inlineStr">
         <is>
           <t>上櫃公司資訊</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr">
+      <c r="F4" s="51" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G4" s="11" t="inlineStr">
+      <c r="G4" s="51" t="inlineStr">
         <is>
           <t>官方一手來源</t>
         </is>
       </c>
-      <c r="H4" s="12" t="inlineStr">
+      <c r="H4" s="48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="51" t="inlineStr">
         <is>
           <t>PRIMARY_COMPANY_IR</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="51" t="inlineStr">
         <is>
           <t>公司 IR 官網</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="51" t="inlineStr">
         <is>
           <t>Primary</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="51" t="inlineStr">
         <is>
           <t>Company IR</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="51" t="inlineStr">
         <is>
           <t>法說會簡報/年報/新聞稿</t>
         </is>
       </c>
-      <c r="F5" s="11" t="inlineStr">
+      <c r="F5" s="51" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G5" s="11" t="inlineStr">
+      <c r="G5" s="51" t="inlineStr">
         <is>
           <t>需確認網址為公司官方網域</t>
         </is>
       </c>
-      <c r="H5" s="12" t="inlineStr">
+      <c r="H5" s="48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="51" t="inlineStr">
         <is>
           <t>SECONDARY_CTEE</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="51" t="inlineStr">
         <is>
           <t>工商時報</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="51" t="inlineStr">
         <is>
           <t>Secondary</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D6" s="51" t="inlineStr">
         <is>
           <t>News</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
+      <c r="E6" s="51" t="inlineStr">
         <is>
           <t>財經新聞</t>
         </is>
       </c>
-      <c r="F6" s="11" t="inlineStr">
+      <c r="F6" s="51" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G6" s="11" t="inlineStr">
+      <c r="G6" s="51" t="inlineStr">
         <is>
           <t>二手來源，需與一手資料交叉檢查</t>
         </is>
       </c>
-      <c r="H6" s="12" t="inlineStr">
+      <c r="H6" s="48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="51" t="inlineStr">
         <is>
           <t>SECONDARY_UDN_ECON</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="51" t="inlineStr">
         <is>
           <t>經濟日報</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="51" t="inlineStr">
         <is>
           <t>Secondary</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="51" t="inlineStr">
         <is>
           <t>News</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="51" t="inlineStr">
         <is>
           <t>財經新聞</t>
         </is>
       </c>
-      <c r="F7" s="11" t="inlineStr">
+      <c r="F7" s="51" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G7" s="11" t="inlineStr">
+      <c r="G7" s="51" t="inlineStr">
         <is>
           <t>二手來源，需標示新聞日期</t>
         </is>
       </c>
-      <c r="H7" s="12" t="inlineStr">
+      <c r="H7" s="48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="51" t="inlineStr">
         <is>
           <t>SECONDARY_MONEYDJ</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="51" t="inlineStr">
         <is>
           <t>MoneyDJ</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="51" t="inlineStr">
         <is>
           <t>Secondary</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="51" t="inlineStr">
         <is>
           <t>News/Data</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="51" t="inlineStr">
         <is>
           <t>財經新聞/產業資料</t>
         </is>
       </c>
-      <c r="F8" s="11" t="inlineStr">
+      <c r="F8" s="51" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G8" s="11" t="inlineStr">
+      <c r="G8" s="51" t="inlineStr">
         <is>
           <t>可作線索，不可替代官方財務數字</t>
         </is>
       </c>
-      <c r="H8" s="12" t="inlineStr">
+      <c r="H8" s="48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="51" t="inlineStr">
         <is>
           <t>SECONDARY_CNA</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="51" t="inlineStr">
         <is>
           <t>中央社</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="51" t="inlineStr">
         <is>
           <t>Secondary</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D9" s="51" t="inlineStr">
         <is>
           <t>News</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="51" t="inlineStr">
         <is>
           <t>新聞</t>
         </is>
       </c>
-      <c r="F9" s="11" t="inlineStr">
+      <c r="F9" s="51" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G9" s="11" t="inlineStr">
+      <c r="G9" s="51" t="inlineStr">
         <is>
           <t>可作事件線索</t>
         </is>
       </c>
-      <c r="H9" s="12" t="inlineStr">
+      <c r="H9" s="48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="51" t="inlineStr">
         <is>
           <t>LOW_SOCIAL</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="51" t="inlineStr">
         <is>
           <t>社群/論壇</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="51" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="51" t="inlineStr">
         <is>
           <t>Social</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="51" t="inlineStr">
         <is>
           <t>討論/傳聞</t>
         </is>
       </c>
-      <c r="F10" s="11" t="inlineStr">
+      <c r="F10" s="51" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G10" s="11" t="inlineStr">
+      <c r="G10" s="51" t="inlineStr">
         <is>
           <t>僅作輿情，不作事實依據</t>
         </is>
       </c>
-      <c r="H10" s="12" t="inlineStr">
+      <c r="H10" s="48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="48" t="inlineStr">
         <is>
           <t>PRIMARY_COMPANY_IR_EN</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="48" t="inlineStr">
         <is>
           <t>Company IR Website</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
+      <c r="C11" s="48" t="inlineStr">
         <is>
           <t>Primary</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="D11" s="48" t="inlineStr">
         <is>
           <t>Company IR</t>
         </is>
       </c>
-      <c r="E11" s="12" t="inlineStr">
+      <c r="E11" s="48" t="inlineStr">
         <is>
           <t>法說會簡報/年報/新聞稿</t>
         </is>
       </c>
-      <c r="F11" s="12" t="inlineStr">
+      <c r="F11" s="48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G11" s="12" t="inlineStr">
+      <c r="G11" s="48" t="inlineStr">
         <is>
           <t>官方公司投資人關係網站；需確認為公司官方網域</t>
         </is>
       </c>
-      <c r="H11" s="12" t="inlineStr">
+      <c r="H11" s="48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="48" t="inlineStr">
         <is>
           <t>PRIMARY_EC_TRANSCRIPT</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="48" t="inlineStr">
         <is>
           <t>Earnings Call Transcript</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C12" s="48" t="inlineStr">
         <is>
           <t>Primary</t>
         </is>
       </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="D12" s="48" t="inlineStr">
         <is>
           <t>Transcript</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="48" t="inlineStr">
         <is>
           <t>法說會逐字稿/問答紀錄</t>
         </is>
       </c>
-      <c r="F12" s="12" t="inlineStr">
+      <c r="F12" s="48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G12" s="12" t="inlineStr">
+      <c r="G12" s="48" t="inlineStr">
         <is>
           <t>若為第三方轉錄，需同時標示轉錄來源與公司法說會日期</t>
         </is>
       </c>
-      <c r="H12" s="12" t="inlineStr">
+      <c r="H12" s="48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="48" t="inlineStr">
         <is>
           <t>PRIMARY_TWSE_ANNOUNCEMENT</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="48" t="inlineStr">
         <is>
           <t>TWSE Announcement</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C13" s="48" t="inlineStr">
         <is>
           <t>Primary</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D13" s="48" t="inlineStr">
         <is>
           <t>TWSE</t>
         </is>
       </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="E13" s="48" t="inlineStr">
         <is>
           <t>上市公司公告/交易所資訊</t>
         </is>
       </c>
-      <c r="F13" s="12" t="inlineStr">
+      <c r="F13" s="48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G13" s="12" t="inlineStr">
+      <c r="G13" s="48" t="inlineStr">
         <is>
           <t>官方一手來源，適合驗證公告與制度資訊</t>
         </is>
       </c>
-      <c r="H13" s="12" t="inlineStr">
+      <c r="H13" s="48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="48" t="inlineStr">
         <is>
           <t>PRIMARY_TPEX_ANNOUNCEMENT</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="48" t="inlineStr">
         <is>
           <t>TPEx Announcement</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="C14" s="48" t="inlineStr">
         <is>
           <t>Primary</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D14" s="48" t="inlineStr">
         <is>
           <t>TPEx</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="48" t="inlineStr">
         <is>
           <t>上櫃公司公告/櫃買資訊</t>
         </is>
       </c>
-      <c r="F14" s="12" t="inlineStr">
+      <c r="F14" s="48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G14" s="12" t="inlineStr">
+      <c r="G14" s="48" t="inlineStr">
         <is>
           <t>官方一手來源，適合驗證上櫃公司公告</t>
         </is>
       </c>
-      <c r="H14" s="12" t="inlineStr">
+      <c r="H14" s="48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="48" t="inlineStr">
+        <is>
+          <t>SECONDARY_YAHOO</t>
+        </is>
+      </c>
+      <c r="B15" s="48" t="inlineStr">
+        <is>
+          <t>YAHOO財經</t>
+        </is>
+      </c>
+      <c r="C15" s="48" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="D15" s="48" t="inlineStr">
+        <is>
+          <t>News/Data</t>
+        </is>
+      </c>
+      <c r="E15" s="48" t="inlineStr">
+        <is>
+          <t>財經新聞/產業資料</t>
+        </is>
+      </c>
+      <c r="F15" s="48" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G15" s="48" t="inlineStr">
+        <is>
+          <t>可作線索，不可替代官方財務數字</t>
+        </is>
+      </c>
+      <c r="H15" s="48" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="48" t="inlineStr">
+        <is>
+          <t>SECONDARY_NEWS_MEDIA</t>
+        </is>
+      </c>
+      <c r="B16" s="48" t="inlineStr">
+        <is>
+          <t>報章雜誌媒體</t>
+        </is>
+      </c>
+      <c r="C16" s="48" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="D16" s="48" t="inlineStr">
+        <is>
+          <t>News/Data</t>
+        </is>
+      </c>
+      <c r="E16" s="48" t="inlineStr">
+        <is>
+          <t>財經新聞/產業資料</t>
+        </is>
+      </c>
+      <c r="F16" s="48" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G16" s="48" t="inlineStr">
+        <is>
+          <t>可作線索，不可替代官方財務數字</t>
+        </is>
+      </c>
+      <c r="H16" s="48" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:H16"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -6336,12 +6437,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="3"/>
-    <col width="96" customWidth="1" min="3" max="3"/>
+    <col width="120" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -6732,6 +6833,23 @@
       <c r="C23" t="inlineStr">
         <is>
           <t>Renamed 10_news_source_whitelist.source_id to source_key for R4 source mapping alignment; added 16_quarter_table covering 2024Q1 through 2026Q4 with fiscal_period/year/quarter/yyyyqq/start_date/end_date/month_keys mapping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="42" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B24" s="42" t="inlineStr">
+        <is>
+          <t>DISCLOSURE_EVENTS_AND_NEWS_SOURCES</t>
+        </is>
+      </c>
+      <c r="C24" s="42" t="inlineStr">
+        <is>
+          <t>2026-06-18 - 04_disclosure_events：改用 event_key 作為 primary key；新增 event_type / event_subtype 分層；補上 major_news 底下的重大訊息子分類；新增或確認 10_news_source_whitelist 中的 SECONDARY_YAHOO 與 SECONDARY_NEWS_MEDIA；目的為支援 R4 metadata tagging、semantic layer filtering 與 R6 citation QA。</t>
         </is>
       </c>
     </row>
@@ -12502,519 +12620,628 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col width="19" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
-    <col width="12" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
-    <col width="20" bestFit="1" customWidth="1" style="1" min="3" max="3"/>
-    <col width="15" bestFit="1" customWidth="1" style="1" min="4" max="4"/>
-    <col width="27" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
-    <col width="10" bestFit="1" customWidth="1" style="1" min="6" max="6"/>
-    <col width="16" bestFit="1" customWidth="1" style="1" min="7" max="7"/>
-    <col width="8.83203125" customWidth="1" style="1" min="8" max="13"/>
+    <col width="28" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
+    <col width="18" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
+    <col width="16" bestFit="1" customWidth="1" style="1" min="3" max="3"/>
+    <col width="20" bestFit="1" customWidth="1" style="1" min="4" max="4"/>
+    <col width="22" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
+    <col width="22" bestFit="1" customWidth="1" style="1" min="6" max="6"/>
+    <col width="28" bestFit="1" customWidth="1" style="1" min="7" max="7"/>
+    <col width="52" customWidth="1" style="1" min="8" max="13"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="58" customWidth="1" min="11" max="11"/>
     <col width="8.83203125" customWidth="1" style="1" min="14" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>event_id</t>
-        </is>
-      </c>
-      <c r="B1" s="22" t="inlineStr">
-        <is>
-          <t>event_name</t>
-        </is>
-      </c>
-      <c r="C1" s="22" t="inlineStr">
+      <c r="A1" s="49" t="inlineStr">
+        <is>
+          <t>event_key</t>
+        </is>
+      </c>
+      <c r="B1" s="49" t="inlineStr">
+        <is>
+          <t>event_type</t>
+        </is>
+      </c>
+      <c r="C1" s="49" t="inlineStr">
+        <is>
+          <t>event_type_name</t>
+        </is>
+      </c>
+      <c r="D1" s="49" t="inlineStr">
+        <is>
+          <t>event_subtype</t>
+        </is>
+      </c>
+      <c r="E1" s="49" t="inlineStr">
+        <is>
+          <t>event_subtype_name</t>
+        </is>
+      </c>
+      <c r="F1" s="49" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="D1" s="22" t="inlineStr">
+      <c r="G1" s="49" t="inlineStr">
         <is>
           <t>source_system</t>
         </is>
       </c>
-      <c r="E1" s="22" t="inlineStr">
+      <c r="H1" s="49" t="inlineStr">
         <is>
           <t>required_fields</t>
         </is>
       </c>
-      <c r="F1" s="22" t="inlineStr">
+      <c r="I1" s="49" t="inlineStr">
         <is>
           <t>severity</t>
         </is>
       </c>
-      <c r="G1" s="23" t="inlineStr">
+      <c r="J1" s="49" t="inlineStr">
         <is>
           <t>demo_relevance</t>
         </is>
       </c>
+      <c r="K1" s="49" t="inlineStr">
+        <is>
+          <t>r6_notes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="48" t="inlineStr">
         <is>
           <t>earnings_call</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="48" t="inlineStr">
+        <is>
+          <t>earnings_call</t>
+        </is>
+      </c>
+      <c r="C2" s="48" t="inlineStr">
         <is>
           <t>法說會</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="D2" s="48" t="inlineStr"/>
+      <c r="E2" s="48" t="inlineStr"/>
+      <c r="F2" s="48" t="inlineStr">
         <is>
           <t>Investor Relations</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>公司IR/公開資訊</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>日期,簡報,逐字稿或摘要,問答重點</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="G2" s="48" t="inlineStr">
+        <is>
+          <t>公司 IR / 公開資訊</t>
+        </is>
+      </c>
+      <c r="H2" s="48" t="inlineStr">
+        <is>
+          <t>日期、期間、公司、簡報、逐字稿或摘要、問答重點</t>
+        </is>
+      </c>
+      <c r="I2" s="48" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="J2" s="48" t="inlineStr">
         <is>
           <t>場景1/3</t>
         </is>
       </c>
+      <c r="K2" s="48" t="inlineStr">
+        <is>
+          <t>第一層事件類型；用於法說會 / earnings call chunks。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>earnings_release</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>財報公告</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="A3" s="48" t="inlineStr">
+        <is>
+          <t>major_news.capital_increase</t>
+        </is>
+      </c>
+      <c r="B3" s="48" t="inlineStr">
+        <is>
+          <t>major_news</t>
+        </is>
+      </c>
+      <c r="C3" s="48" t="inlineStr">
+        <is>
+          <t>重大訊息</t>
+        </is>
+      </c>
+      <c r="D3" s="48" t="inlineStr">
+        <is>
+          <t>capital_increase</t>
+        </is>
+      </c>
+      <c r="E3" s="48" t="inlineStr">
+        <is>
+          <t>增資</t>
+        </is>
+      </c>
+      <c r="F3" s="48" t="inlineStr">
+        <is>
+          <t>Disclosure</t>
+        </is>
+      </c>
+      <c r="G3" s="48" t="inlineStr">
+        <is>
+          <t>MOPS</t>
+        </is>
+      </c>
+      <c r="H3" s="48" t="inlineStr">
+        <is>
+          <t>金額、股數、用途、價格、稀釋影響</t>
+        </is>
+      </c>
+      <c r="I3" s="48" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J3" s="48" t="inlineStr">
+        <is>
+          <t>場景2</t>
+        </is>
+      </c>
+      <c r="K3" s="48" t="inlineStr">
+        <is>
+          <t>重大訊息子分類；用於資本市場事件。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="48" t="inlineStr">
+        <is>
+          <t>major_news.capital_reduction</t>
+        </is>
+      </c>
+      <c r="B4" s="48" t="inlineStr">
+        <is>
+          <t>major_news</t>
+        </is>
+      </c>
+      <c r="C4" s="48" t="inlineStr">
+        <is>
+          <t>重大訊息</t>
+        </is>
+      </c>
+      <c r="D4" s="48" t="inlineStr">
+        <is>
+          <t>capital_reduction</t>
+        </is>
+      </c>
+      <c r="E4" s="48" t="inlineStr">
+        <is>
+          <t>減資</t>
+        </is>
+      </c>
+      <c r="F4" s="48" t="inlineStr">
+        <is>
+          <t>Disclosure</t>
+        </is>
+      </c>
+      <c r="G4" s="48" t="inlineStr">
+        <is>
+          <t>MOPS</t>
+        </is>
+      </c>
+      <c r="H4" s="48" t="inlineStr">
+        <is>
+          <t>原因、金額、比例、基準日、對股東影響</t>
+        </is>
+      </c>
+      <c r="I4" s="48" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J4" s="48" t="inlineStr">
+        <is>
+          <t>場景2</t>
+        </is>
+      </c>
+      <c r="K4" s="48" t="inlineStr">
+        <is>
+          <t>重大訊息子分類；需注意是否涉及彌補虧損或現金減資。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="48" t="inlineStr">
+        <is>
+          <t>major_news.share_buyback</t>
+        </is>
+      </c>
+      <c r="B5" s="48" t="inlineStr">
+        <is>
+          <t>major_news</t>
+        </is>
+      </c>
+      <c r="C5" s="48" t="inlineStr">
+        <is>
+          <t>重大訊息</t>
+        </is>
+      </c>
+      <c r="D5" s="48" t="inlineStr">
+        <is>
+          <t>share_buyback</t>
+        </is>
+      </c>
+      <c r="E5" s="48" t="inlineStr">
+        <is>
+          <t>庫藏股</t>
+        </is>
+      </c>
+      <c r="F5" s="48" t="inlineStr">
+        <is>
+          <t>Disclosure</t>
+        </is>
+      </c>
+      <c r="G5" s="48" t="inlineStr">
+        <is>
+          <t>MOPS</t>
+        </is>
+      </c>
+      <c r="H5" s="48" t="inlineStr">
+        <is>
+          <t>買回目的、區間、股數、價格上限</t>
+        </is>
+      </c>
+      <c r="I5" s="48" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J5" s="48" t="inlineStr">
+        <is>
+          <t>場景2</t>
+        </is>
+      </c>
+      <c r="K5" s="48" t="inlineStr">
+        <is>
+          <t>重大訊息子分類；避免被誤判為投資建議。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="48" t="inlineStr">
+        <is>
+          <t>major_news.merger</t>
+        </is>
+      </c>
+      <c r="B6" s="48" t="inlineStr">
+        <is>
+          <t>major_news</t>
+        </is>
+      </c>
+      <c r="C6" s="48" t="inlineStr">
+        <is>
+          <t>重大訊息</t>
+        </is>
+      </c>
+      <c r="D6" s="48" t="inlineStr">
+        <is>
+          <t>merger</t>
+        </is>
+      </c>
+      <c r="E6" s="48" t="inlineStr">
+        <is>
+          <t>併購</t>
+        </is>
+      </c>
+      <c r="F6" s="48" t="inlineStr">
+        <is>
+          <t>Disclosure</t>
+        </is>
+      </c>
+      <c r="G6" s="48" t="inlineStr">
+        <is>
+          <t>MOPS</t>
+        </is>
+      </c>
+      <c r="H6" s="48" t="inlineStr">
+        <is>
+          <t>交易對象、價格、支付方式、股權比例</t>
+        </is>
+      </c>
+      <c r="I6" s="48" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J6" s="48" t="inlineStr">
+        <is>
+          <t>場景2</t>
+        </is>
+      </c>
+      <c r="K6" s="48" t="inlineStr">
+        <is>
+          <t>重大訊息子分類；包含合併、收購、股份轉換等。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="48" t="inlineStr">
+        <is>
+          <t>major_news.asset_disposal</t>
+        </is>
+      </c>
+      <c r="B7" s="48" t="inlineStr">
+        <is>
+          <t>major_news</t>
+        </is>
+      </c>
+      <c r="C7" s="48" t="inlineStr">
+        <is>
+          <t>重大訊息</t>
+        </is>
+      </c>
+      <c r="D7" s="48" t="inlineStr">
+        <is>
+          <t>asset_disposal</t>
+        </is>
+      </c>
+      <c r="E7" s="48" t="inlineStr">
+        <is>
+          <t>處分長期投資 / 資產</t>
+        </is>
+      </c>
+      <c r="F7" s="48" t="inlineStr">
+        <is>
+          <t>Disclosure</t>
+        </is>
+      </c>
+      <c r="G7" s="48" t="inlineStr">
+        <is>
+          <t>MOPS</t>
+        </is>
+      </c>
+      <c r="H7" s="48" t="inlineStr">
+        <is>
+          <t>處分標的、交易對手、價格、帳列金額</t>
+        </is>
+      </c>
+      <c r="I7" s="48" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J7" s="48" t="inlineStr">
+        <is>
+          <t>場景2</t>
+        </is>
+      </c>
+      <c r="K7" s="48" t="inlineStr">
+        <is>
+          <t>重大訊息子分類；可協助排除非營運性損益混淆。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="48" t="inlineStr">
+        <is>
+          <t>major_news.new_factory</t>
+        </is>
+      </c>
+      <c r="B8" s="48" t="inlineStr">
+        <is>
+          <t>major_news</t>
+        </is>
+      </c>
+      <c r="C8" s="48" t="inlineStr">
+        <is>
+          <t>重大訊息</t>
+        </is>
+      </c>
+      <c r="D8" s="48" t="inlineStr">
+        <is>
+          <t>new_factory</t>
+        </is>
+      </c>
+      <c r="E8" s="48" t="inlineStr">
+        <is>
+          <t>擴廠</t>
+        </is>
+      </c>
+      <c r="F8" s="48" t="inlineStr">
+        <is>
+          <t>Disclosure</t>
+        </is>
+      </c>
+      <c r="G8" s="48" t="inlineStr">
+        <is>
+          <t>MOPS / 公司公告 / 新聞</t>
+        </is>
+      </c>
+      <c r="H8" s="48" t="inlineStr">
+        <is>
+          <t>地點、投資金額、產能、時程、客戶</t>
+        </is>
+      </c>
+      <c r="I8" s="48" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J8" s="48" t="inlineStr">
+        <is>
+          <t>場景3</t>
+        </is>
+      </c>
+      <c r="K8" s="48" t="inlineStr">
+        <is>
+          <t>重大訊息子分類；與產能、供應鏈、AI 需求題可能相關。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="48" t="inlineStr">
+        <is>
+          <t>major_news.others</t>
+        </is>
+      </c>
+      <c r="B9" s="48" t="inlineStr">
+        <is>
+          <t>major_news</t>
+        </is>
+      </c>
+      <c r="C9" s="48" t="inlineStr">
+        <is>
+          <t>重大訊息</t>
+        </is>
+      </c>
+      <c r="D9" s="48" t="inlineStr">
+        <is>
+          <t>others</t>
+        </is>
+      </c>
+      <c r="E9" s="48" t="inlineStr">
+        <is>
+          <t>其他重大訊息</t>
+        </is>
+      </c>
+      <c r="F9" s="48" t="inlineStr">
+        <is>
+          <t>Disclosure</t>
+        </is>
+      </c>
+      <c r="G9" s="48" t="inlineStr">
+        <is>
+          <t>MOPS</t>
+        </is>
+      </c>
+      <c r="H9" s="48" t="inlineStr">
+        <is>
+          <t>事件日期、主旨、說明、對公司影響</t>
+        </is>
+      </c>
+      <c r="I9" s="48" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J9" s="48" t="inlineStr">
+        <is>
+          <t>場景2</t>
+        </is>
+      </c>
+      <c r="K9" s="48" t="inlineStr">
+        <is>
+          <t>無法歸入上述 subtype 時使用；後續可依測試結果再拆細。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="48" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="B10" s="48" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C10" s="48" t="inlineStr">
+        <is>
+          <t>新聞</t>
+        </is>
+      </c>
+      <c r="D10" s="48" t="inlineStr"/>
+      <c r="E10" s="48" t="inlineStr"/>
+      <c r="F10" s="48" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="G10" s="48" t="inlineStr">
+        <is>
+          <t>新聞 / 公開資訊</t>
+        </is>
+      </c>
+      <c r="H10" s="48" t="inlineStr">
+        <is>
+          <t>日期、來源、公司、事件摘要、關聯主題</t>
+        </is>
+      </c>
+      <c r="I10" s="48" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J10" s="48" t="inlineStr">
+        <is>
+          <t>場景3</t>
+        </is>
+      </c>
+      <c r="K10" s="48" t="inlineStr">
+        <is>
+          <t>第一層事件類型；非 MOPS 重大訊息，需注意來源可信度。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="48" t="inlineStr">
+        <is>
+          <t>monthly_revenue</t>
+        </is>
+      </c>
+      <c r="B11" s="48" t="inlineStr">
+        <is>
+          <t>monthly_revenue</t>
+        </is>
+      </c>
+      <c r="C11" s="48" t="inlineStr">
+        <is>
+          <t>月營收</t>
+        </is>
+      </c>
+      <c r="D11" s="48" t="inlineStr"/>
+      <c r="E11" s="48" t="inlineStr"/>
+      <c r="F11" s="48" t="inlineStr">
         <is>
           <t>Financial</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>MOPS/公司公告</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>期間,營收,毛利率,EPS,管理層說明</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G11" s="48" t="inlineStr">
+        <is>
+          <t>MOPS / 公司公告</t>
+        </is>
+      </c>
+      <c r="H11" s="48" t="inlineStr">
+        <is>
+          <t>年月、本月營收、年增率、月增率、累計營收</t>
+        </is>
+      </c>
+      <c r="I11" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>場景1</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>monthly_revenue</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>月營收公告</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Financial</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>MOPS</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>年月,本月營收,去年同期,年增率,累計營收</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="J11" s="48" t="inlineStr">
         <is>
           <t>投研基礎</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>dividend</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>股利公告</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Shareholder</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>MOPS/董事會</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>每股現金股利,股票股利,除權息日,發放日</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>board_meeting</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>董事會</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>MOPS</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>開會日期,決議事項,影響說明</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>場景2</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>material_info</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>重大訊息</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Disclosure</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>MOPS</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>事實發生日,主旨,說明,對公司影響</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>場景2</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>capital_increase</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>增資</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Capital Market</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>MOPS</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>金額,股數,用途,價格,稀釋影響</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>capital_reduction</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>減資</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Capital Market</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>MOPS</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>原因,金額,比例,基準日,對股東影響</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>share_buyback</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>庫藏股</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Shareholder</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>MOPS</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>買回目的,區間,股數,價格上限</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>merger</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>併購</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>MOPS</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>交易對象,價格,支付方式,股權比例,綜效</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>asset_disposal</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>處分長期投資/資產</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>MOPS</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>處分標的,交易對手,價格,帳列金額,損益,未來影響</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>場景2</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>new_factory</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>擴廠</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Operations</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>公司公告/新聞</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>地點,投資金額,產能,時程,客戶</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>場景3</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>guidance</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>財測發布/展望</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>Management</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>法說會/公告</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>期間,假設,區間,主要變因</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>紅隊</t>
+      <c r="K11" s="48" t="inlineStr">
+        <is>
+          <t>第一層事件類型；用於月營收公告，避免混入法說會題。</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K11"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs(r6): update finance metric dictionary
</commit_message>
<xml_diff>
--- a/docs/r6/ontology/Ontology_V1.xlsx
+++ b/docs/r6/ontology/Ontology_V1.xlsx
@@ -338,7 +338,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -489,6 +489,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6437,7 +6446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6850,6 +6859,23 @@
       <c r="C24" s="42" t="inlineStr">
         <is>
           <t>2026-06-18 - 04_disclosure_events：改用 event_key 作為 primary key；新增 event_type / event_subtype 分層；補上 major_news 底下的重大訊息子分類；新增或確認 10_news_source_whitelist 中的 SECONDARY_YAHOO 與 SECONDARY_NEWS_MEDIA；目的為支援 R4 metadata tagging、semantic layer filtering 與 R6 citation QA。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="54" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B25" s="54" t="inlineStr">
+        <is>
+          <t>FINANCIAL_METRIC_ENUM_UPDATE_2026-06-23</t>
+        </is>
+      </c>
+      <c r="C25" s="54" t="inlineStr">
+        <is>
+          <t>Added finance metric IDs pretax_income, operating_expense, revenue_delta, revenue_yoy; clarified revenue_yoy vs ytd_yoy.</t>
         </is>
       </c>
     </row>
@@ -9627,7 +9653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="18" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -10929,6 +10955,234 @@
       <c r="K23" t="inlineStr">
         <is>
           <t>mops_monthly_revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="52" t="inlineStr">
+        <is>
+          <t>pretax_income</t>
+        </is>
+      </c>
+      <c r="B24" s="52" t="inlineStr">
+        <is>
+          <t>稅前淨利</t>
+        </is>
+      </c>
+      <c r="C24" s="52" t="inlineStr">
+        <is>
+          <t>稅前利益,所得稅前損益,pretax profit</t>
+        </is>
+      </c>
+      <c r="D24" s="52" t="inlineStr">
+        <is>
+          <t>獲利</t>
+        </is>
+      </c>
+      <c r="E24" s="52" t="inlineStr">
+        <is>
+          <t>新台幣千元</t>
+        </is>
+      </c>
+      <c r="F24" s="52" t="inlineStr">
+        <is>
+          <t>所得稅前損益，用於觀察公司稅前獲利能力。</t>
+        </is>
+      </c>
+      <c r="G24" s="52" t="inlineStr">
+        <is>
+          <t>財報/IFRS</t>
+        </is>
+      </c>
+      <c r="H24" s="52" t="inlineStr">
+        <is>
+          <t>季/年</t>
+        </is>
+      </c>
+      <c r="I24" s="52" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J24" s="52" t="inlineStr">
+        <is>
+          <t>不等同於 net_income，需注意是否為稅前數。</t>
+        </is>
+      </c>
+      <c r="K24" s="53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="52" t="inlineStr">
+        <is>
+          <t>operating_expense</t>
+        </is>
+      </c>
+      <c r="B25" s="52" t="inlineStr">
+        <is>
+          <t>營業費用</t>
+        </is>
+      </c>
+      <c r="C25" s="52" t="inlineStr">
+        <is>
+          <t>營業費用合計,OPEX,operating expenses</t>
+        </is>
+      </c>
+      <c r="D25" s="52" t="inlineStr">
+        <is>
+          <t>獲利</t>
+        </is>
+      </c>
+      <c r="E25" s="52" t="inlineStr">
+        <is>
+          <t>新台幣千元</t>
+        </is>
+      </c>
+      <c r="F25" s="52" t="inlineStr">
+        <is>
+          <t>營業活動相關費用，通常包含推銷費用、管理費用、研發費用等。</t>
+        </is>
+      </c>
+      <c r="G25" s="52" t="inlineStr">
+        <is>
+          <t>財報/IFRS</t>
+        </is>
+      </c>
+      <c r="H25" s="52" t="inlineStr">
+        <is>
+          <t>季/年</t>
+        </is>
+      </c>
+      <c r="I25" s="52" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J25" s="52" t="inlineStr">
+        <is>
+          <t>若資料來源拆分 SG&amp;A / R&amp;D，需確認是否加總為營業費用。</t>
+        </is>
+      </c>
+      <c r="K25" s="53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="40" t="inlineStr">
+        <is>
+          <t>revenue_delta</t>
+        </is>
+      </c>
+      <c r="B26" s="40" t="inlineStr">
+        <is>
+          <t>營收增減金額</t>
+        </is>
+      </c>
+      <c r="C26" s="40" t="inlineStr">
+        <is>
+          <t>營收增減,營收差額,revenue change</t>
+        </is>
+      </c>
+      <c r="D26" s="40" t="inlineStr">
+        <is>
+          <t>成長</t>
+        </is>
+      </c>
+      <c r="E26" s="40" t="inlineStr">
+        <is>
+          <t>TWD_thousand</t>
+        </is>
+      </c>
+      <c r="F26" s="40" t="inlineStr">
+        <is>
+          <t>本期營收與比較基期營收的差額，可用於月營收、季度營收或年度營收比較。</t>
+        </is>
+      </c>
+      <c r="G26" s="40" t="inlineStr">
+        <is>
+          <t>計算指標</t>
+        </is>
+      </c>
+      <c r="H26" s="40" t="inlineStr">
+        <is>
+          <t>月/季/年</t>
+        </is>
+      </c>
+      <c r="I26" s="40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J26" s="40" t="inlineStr">
+        <is>
+          <t>需搭配 comparison_base，例如 MoM、YoY、QoQ 或指定比較期間。</t>
+        </is>
+      </c>
+      <c r="K26" s="40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="40" t="inlineStr">
+        <is>
+          <t>revenue_yoy</t>
+        </is>
+      </c>
+      <c r="B27" s="40" t="inlineStr">
+        <is>
+          <t>營收年增率</t>
+        </is>
+      </c>
+      <c r="C27" s="40" t="inlineStr">
+        <is>
+          <t>單期營收年增率,revenue YoY</t>
+        </is>
+      </c>
+      <c r="D27" s="40" t="inlineStr">
+        <is>
+          <t>成長</t>
+        </is>
+      </c>
+      <c r="E27" s="40" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F27" s="40" t="inlineStr">
+        <is>
+          <t>(本期營收 - 去年同期營收) / 去年同期營收</t>
+        </is>
+      </c>
+      <c r="G27" s="40" t="inlineStr">
+        <is>
+          <t>計算指標</t>
+        </is>
+      </c>
+      <c r="H27" s="40" t="inlineStr">
+        <is>
+          <t>月/季/年</t>
+        </is>
+      </c>
+      <c r="I27" s="40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J27" s="40" t="inlineStr">
+        <is>
+          <t>revenue_yoy 是單期營收年增率；不要和 ytd_yoy 混用。</t>
+        </is>
+      </c>
+      <c r="K27" s="40" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
     </row>

</xml_diff>